<commit_message>
Add 14 products: Solaray (7), NOW NAC/CoQ10 (3), ECOVITA magnesium/ALA/5-HTP (4)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -772,7 +772,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>195 товаров · 13 брендов · 19 категорий</t>
+          <t>209 товаров · 13 брендов · 19 категорий</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE196"/>
+  <dimension ref="A1:AE210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.05"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -24619,6 +24619,1708 @@
         </is>
       </c>
       <c r="Y196" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>solaray-vitamin-c-500</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>solaray-buffered-vitamin-c-bioflavonoids-500mg-100-vegcaps</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Solaray Buffered Vitamin C с биофлавоноидами 500 мг, 100 растительных капсул</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Solaray Buffered Vitamin C bioflavonoidlar bilan 500 mg, 100 oʻsimlik kapsulasi</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Витамины</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Иммунитет</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Капсулы</t>
+        </is>
+      </c>
+      <c r="I197" t="n">
+        <v>500</v>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="K197" t="n">
+        <v>100</v>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>Забуференный витамин C 500 мг с биофлавоноидным концентратом для иммунитета.</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>Immunitet uchun bioflavonoid konsentratli buferlangan vitamin C 500 mg.</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>Solaray Buffered Vitamin C — витамин C в забуференной (мягкой для желудка) форме с биофлавоноидным концентратом из лимона, рутином, гесперидином и основой из шиповника и ацеролы. Укрепляет иммунитет и работает как антиоксидант. Веганский продукт, подтверждена эффективность лабораторными исследованиями.</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>Solaray Buffered Vitamin C — limondan olingan bioflavonoid konsentrati, rutin, gesperidin hamda na’matak va asserola asosi bilan buferlangan (oshqozon uchun yumshoq) shakldagi vitamin C. Immunitetni mustahkamlaydi va antioksidant sifatida ishlaydi. Vegan mahsulot, samaradorligi laboratoriya tadqiqotlari bilan tasdiqlangan.</t>
+        </is>
+      </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>1 капсула содержит: витамин C (аскорбиновая кислота) — 500 мг; кальций (карбонат кальция) — 20 мг; магний (оксид магния) — 37 мг; основа для поддержки витамина C (шиповник, ацерола) — 95 мг; концентрат биофлавоноидов (из лимона) — 100 мг; концентрат рутина — 50 мг; концентрат гесперидина — 25 мг; капсула из растительной целлюлозы, стеарат магния, акация</t>
+        </is>
+      </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>1 kapsula tarkibida: vitamin C (askorbin kislotasi) — 500 mg; kaltsiy (kaltsiy karbonat) — 20 mg; magniy (magniy oksid) — 37 mg; vitamin C ni qoʻllab-quvvatlovchi asos (na’matak, asserola) — 95 mg; bioflavonoidlar konsentrati (limondan) — 100 mg; rutin konsentrati — 50 mg; gesperidin konsentrati — 25 mg; oʻsimlik sellyulozasi kapsulasi, magniy stearati, akatsiya</t>
+        </is>
+      </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>Взрослым — по 1 растительной капсуле в день во время еды или запивая стаканом воды.</t>
+        </is>
+      </c>
+      <c r="S197" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 1 oʻsimlik kapsulasi, ovqat vaqtida yoki bir stakan suv bilan.</t>
+        </is>
+      </c>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>Не использовать, если защитная плёнка повреждена или отсутствует. Хранить в недоступном для детей месте, в сухом и прохладном месте. Перед началом применения проконсультируйтесь с врачом.</t>
+        </is>
+      </c>
+      <c r="U197" t="inlineStr">
+        <is>
+          <t>Himoya pardasi shikastlangan yoki yoʻq boʻlsa, ishlatmang. Bolalar yeta olmaydigan, quruq va salqin joyda saqlang. Qoʻllashdan oldin shifokor bilan maslahatlashing.</t>
+        </is>
+      </c>
+      <c r="V197" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="W197" t="inlineStr">
+        <is>
+          <t>США</t>
+        </is>
+      </c>
+      <c r="X197" t="inlineStr">
+        <is>
+          <t>images/solaray-vitamin-c-buffered-500.jpg</t>
+        </is>
+      </c>
+      <c r="Y197" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>solaray-chromium-500</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>solaray-chromium-picolinate-500mcg-60-tabs</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Solaray Chromium Picolinate 500 мкг, 60 таблеток</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Solaray Chromium Picolinate 500 mkg, 60 tabletka</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Минералы</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Таблетки</t>
+        </is>
+      </c>
+      <c r="I198" t="n">
+        <v>500</v>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>мкг</t>
+        </is>
+      </c>
+      <c r="K198" t="n">
+        <v>60</v>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>Пиколинат хрома 500 мкг для поддержки здорового уровня глюкозы в крови.</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>Qondagi glyukoza darajasini sogʻlom saqlash uchun xrom pikolinat 500 mkg.</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>Solaray Chromium Picolinate — хром в предпочтительной трёхвалентной форме (пиколинат). Предназначен для питательной поддержки здорового уровня глюкозы в крови. Эффективность подтверждена результатами лабораторных исследований.</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>Solaray Chromium Picolinate — afzal koʻriladigan uch valentli shakldagi (pikolinat) xrom. Qondagi glyukoza darajasini sogʻlom saqlashga oziqaviy yordam berish uchun moʻljallangan. Samaradorligi laboratoriya tadqiqotlari bilan tasdiqlangan.</t>
+        </is>
+      </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>1 таблетка содержит: хром (из пиколината хрома) — 500 мкг; целлюлоза, стеариновая кислота, кроскармеллоза натрия, стеарат магния</t>
+        </is>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>1 tabletka tarkibida: xrom (xrom pikolinatdan) — 500 mkg; sellyuloza, stearin kislotasi, natriy kroskarmelloza, magniy stearati</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>Взрослым — по 1 таблетке в день во время еды или запивая стаканом воды.</t>
+        </is>
+      </c>
+      <c r="S198" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 1 tabletka, ovqat vaqtida yoki bir stakan suv bilan.</t>
+        </is>
+      </c>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>Не использовать, если защитная плёнка повреждена или отсутствует. Хранить в недоступном для детей месте, в сухом и прохладном месте. Перед началом применения проконсультируйтесь с врачом.</t>
+        </is>
+      </c>
+      <c r="U198" t="inlineStr">
+        <is>
+          <t>Himoya pardasi shikastlangan yoki yoʻq boʻlsa, ishlatmang. Bolalar yeta olmaydigan, quruq va salqin joyda saqlang. Qoʻllashdan oldin shifokor bilan maslahatlashing.</t>
+        </is>
+      </c>
+      <c r="V198" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="W198" t="inlineStr">
+        <is>
+          <t>США</t>
+        </is>
+      </c>
+      <c r="X198" t="inlineStr">
+        <is>
+          <t>images/solaray-chromium-picolinate-500.jpg</t>
+        </is>
+      </c>
+      <c r="Y198" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>solaray-selenium-200-100</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>solaray-high-potency-selenium-200mcg-100-vegcaps</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Solaray High Potency Selenium 200 мкг, 100 растительных капсул</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Solaray High Potency Selenium 200 mkg, 100 oʻsimlik kapsulasi</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Минералы</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Антиоксиданты</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Капсулы</t>
+        </is>
+      </c>
+      <c r="I199" t="n">
+        <v>200</v>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>мкг</t>
+        </is>
+      </c>
+      <c r="K199" t="n">
+        <v>100</v>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>Высокоэффективный селен 200 мкг из селеновых дрожжей — антиоксидантная защита.</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>Selenli xamirturushdan olingan yuqori samarali selen 200 mkg — antioksidant himoya.</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>Solaray High Potency Selenium — селен из органически связанных селеновых дрожжей. Незаменимый микроэлемент, обеспечивающий антиоксидантную защиту. Эффективность подтверждена результатами лабораторных исследований.</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>Solaray High Potency Selenium — organik bogʻlangan selenli xamirturushdan olingan selen. Antioksidant himoyani taʼminlovchi muhim mikroelement. Samaradorligi laboratoriya tadqiqotlari bilan tasdiqlangan.</t>
+        </is>
+      </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>1 капсула содержит: селен (из органически связанных селеновых дрожжей) — 200 мкг; пищевые дрожжи, растительная целлюлоза (капсула), стеарат магния</t>
+        </is>
+      </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>1 kapsula tarkibida: selen (organik bogʻlangan selenli xamirturushdan) — 200 mkg; oziq-ovqat xamirturushi, oʻsimlik sellyulozasi (kapsula), magniy stearati</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>Взрослым — по 1 вегетарианской капсуле в день во время еды или запивая стаканом воды.</t>
+        </is>
+      </c>
+      <c r="S199" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 1 vegetarian kapsula, ovqat vaqtida yoki bir stakan suv bilan.</t>
+        </is>
+      </c>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>Хранить плотно закрытым в прохладном, сухом месте, в недоступном для детей месте. Содержит дрожжи.</t>
+        </is>
+      </c>
+      <c r="U199" t="inlineStr">
+        <is>
+          <t>Zich yopilgan holda, salqin va quruq, bolalar yeta olmaydigan joyda saqlang. Tarkibida xamirturush bor.</t>
+        </is>
+      </c>
+      <c r="V199" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="W199" t="inlineStr">
+        <is>
+          <t>США</t>
+        </is>
+      </c>
+      <c r="X199" t="inlineStr">
+        <is>
+          <t>images/solaray-high-potency-selenium-200.jpg</t>
+        </is>
+      </c>
+      <c r="Y199" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>solaray-zinc-50</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>solaray-zinc-50mg-100-vegcaps</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Solaray Zinc 50 мг, 100 растительных капсул</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Solaray Zinc 50 mg, 100 oʻsimlik kapsulasi</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Минералы</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Иммунитет</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Капсулы</t>
+        </is>
+      </c>
+      <c r="I200" t="n">
+        <v>50</v>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="K200" t="n">
+        <v>100</v>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>Аминокислотный хелат цинка 50 мг для иммунитета, кожи и работы клеток.</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>Immunitet, teri va hujayralar ishi uchun aminokislotali rux xelati 50 mg.</t>
+        </is>
+      </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>Solaray Zinc — 50 мг цинка в виде аминокислотного хелата для лучшего усвоения. Цинк участвует более чем в 100 ферментативных реакциях, необходим для иммунной системы, здоровья кожи и работы клеток и не накапливается в организме. Веганский продукт.</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>Solaray Zinc — yaxshi oʻzlashishi uchun aminokislotali xelat shaklidagi 50 mg rux. Rux 100 dan ortiq fermentativ reaksiyada ishtirok etadi, immun tizimi, teri salomatligi va hujayralar ishi uchun zarur va organizmda toʻplanmaydi. Vegan mahsulot.</t>
+        </is>
+      </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>1 капсула содержит: цинк (из комплекса аминокислотного хелата цинка) — 50 мг; семена тыквы (Cucurbita pepo) — 50 мг; концентрат цельного риса, капсула из растительной целлюлозы, целлюлоза, смесь экстрактов органического риса, диоксид кремния</t>
+        </is>
+      </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>1 kapsula tarkibida: rux (rux aminokislotali xelat kompleksidan) — 50 mg; qovoq (Cucurbita pepo) urugʻi — 50 mg; butun guruch konsentrati, oʻsimlik sellyulozasi kapsulasi, sellyuloza, organik guruch ekstraktlari aralashmasi, kremniy dioksidi</t>
+        </is>
+      </c>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>Взрослым — по 1 растительной капсуле в день во время еды или запивая стаканом воды.</t>
+        </is>
+      </c>
+      <c r="S200" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 1 oʻsimlik kapsulasi, ovqat vaqtida yoki bir stakan suv bilan.</t>
+        </is>
+      </c>
+      <c r="T200" t="inlineStr">
+        <is>
+          <t>Не использовать, если защитная плёнка повреждена или отсутствует. Хранить в недоступном для детей месте, в сухом и прохладном месте. Перед началом применения проконсультируйтесь с врачом. Длительное применение может повлиять на статус меди — возможно, потребуется дополнительный приём меди.</t>
+        </is>
+      </c>
+      <c r="U200" t="inlineStr">
+        <is>
+          <t>Himoya pardasi shikastlangan yoki yoʻq boʻlsa, ishlatmang. Bolalar yeta olmaydigan, quruq va salqin joyda saqlang. Qoʻllashdan oldin shifokor bilan maslahatlashing. Uzoq muddat qabul qilish mis holatiga taʼsir qilishi mumkin — qoʻshimcha mis qabul qilish zarur boʻlishi mumkin.</t>
+        </is>
+      </c>
+      <c r="V200" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="W200" t="inlineStr">
+        <is>
+          <t>США</t>
+        </is>
+      </c>
+      <c r="X200" t="inlineStr">
+        <is>
+          <t>images/solaray-zinc-50.jpg</t>
+        </is>
+      </c>
+      <c r="Y200" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>solaray-iron-50</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>solaray-iron-50mg-60-vegcaps</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Solaray Iron 50 мг, 60 растительных капсул</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Solaray Iron 50 mg, 60 oʻsimlik kapsulasi</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Железо</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Минералы</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Капсулы</t>
+        </is>
+      </c>
+      <c r="I201" t="n">
+        <v>50</v>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="K201" t="n">
+        <v>60</v>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>Аминокислотный хелат железа 50 мг — усвояемая форма для кровообращения.</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>Qon aylanishi uchun yaxshi oʻzlashadigan aminokislotali temir xelati 50 mg.</t>
+        </is>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>Solaray Iron — железо, вступившее в реакцию с аспарагиновой кислотой, концентратом цельного риса и лимонной кислотой для создания более усваиваемого хелатного комплекса. Железо — жизненно важная часть красных кровяных телец; поддерживает кровообращение и здоровье сердечно-сосудистой системы.</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>Solaray Iron — aspartik kislota, butun guruch konsentrati va limon kislotasi bilan reaksiyaga kirishib, yaxshiroq oʻzlashadigan xelat kompleksi hosil qilgan temir. Temir — qizil qon tanachalarining muhim qismi; qon aylanishi va yurak-qon tomir tizimi salomatligini qoʻllab-quvvatlaydi.</t>
+        </is>
+      </c>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t>1 капсула содержит: железо (из комплекса аминокислотного хелата железа) — 50 мг; травяная основа (листья петрушки, рисовая мука, корень щавеля), капсула из растительной целлюлозы, аскорбил пальмитат</t>
+        </is>
+      </c>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>1 kapsula tarkibida: temir (temirning aminokislotali xelat kompleksidan) — 50 mg; oʻsimlik asosi (petrushka bargi, guruch uni, shovul ildizi), oʻsimlik sellyulozasi kapsulasi, askorbil palmitat</t>
+        </is>
+      </c>
+      <c r="R201" t="inlineStr">
+        <is>
+          <t>Взрослым — по 1 растительной капсуле в день во время еды или запивая стаканом воды.</t>
+        </is>
+      </c>
+      <c r="S201" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 1 oʻsimlik kapsulasi, ovqat vaqtida yoki bir stakan suv bilan.</t>
+        </is>
+      </c>
+      <c r="T201" t="inlineStr">
+        <is>
+          <t>Не использовать, если защитная плёнка повреждена или отсутствует. Хранить в недоступном для детей месте, в сухом и прохладном месте. Перед началом применения проконсультируйтесь с врачом. Не предназначено для лиц младше 18 лет. Случайная передозировка препаратов железа — основная причина отравлений со смертельным исходом у детей до 6 лет; при передозировке немедленно обратитесь к врачу или в токсикологический центр.</t>
+        </is>
+      </c>
+      <c r="U201" t="inlineStr">
+        <is>
+          <t>Himoya pardasi shikastlangan yoki yoʻq boʻlsa, ishlatmang. Bolalar yeta olmaydigan, quruq va salqin joyda saqlang. Qoʻllashdan oldin shifokor bilan maslahatlashing. 18 yoshgacha boʻlganlar uchun moʻljallanmagan. Temir preparatlarining tasodifiy ortiqcha dozasi 6 yoshgacha boʻlgan bolalarda oʻlimga olib keluvchi zaharlanishning asosiy sababidir; ortiqcha doza qabul qilinganda darhol shifokorga yoki toksikologiya markaziga murojaat qiling.</t>
+        </is>
+      </c>
+      <c r="V201" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="W201" t="inlineStr">
+        <is>
+          <t>США</t>
+        </is>
+      </c>
+      <c r="X201" t="inlineStr">
+        <is>
+          <t>images/solaray-iron-50.jpg</t>
+        </is>
+      </c>
+      <c r="Y201" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>solaray-inositol-500</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>solaray-inositol-500mg-100-vegcaps</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Solaray Inositol 500 мг, 100 растительных капсул</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Solaray Inositol 500 mg, 100 oʻsimlik kapsulasi</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Витамины</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Нервная система и сон</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Капсулы</t>
+        </is>
+      </c>
+      <c r="I202" t="n">
+        <v>500</v>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="K202" t="n">
+        <v>100</v>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>Инозитол 500 мг для здоровья на клеточном уровне.</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>Hujayra darajasidagi salomatlik uchun inozitol 500 mg.</t>
+        </is>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>Solaray Inositol — инозитол, питательное вещество, которое вырабатывается в организме, а также содержится в растениях и продуктах животного происхождения. Обеспечивает питательную поддержку клеточного здоровья и хорошего самочувствия. Вегетарианский продукт.</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>Solaray Inositol — organizmda ishlab chiqariladigan hamda oʻsimlik va hayvon mahsulotlarida uchraydigan oziq modda inozitol. Hujayra salomatligi va yaxshi kayfiyatga oziqaviy yordam beradi. Vegetarian mahsulot.</t>
+        </is>
+      </c>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t>1 капсула содержит: инозитол — 500 мг; капсула из растительной целлюлозы, концентрат цельного риса, экстракт органических рисовых отрубей, диоксид кремния</t>
+        </is>
+      </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>1 kapsula tarkibida: inozitol — 500 mg; oʻsimlik sellyulozasi kapsulasi, butun guruch konsentrati, organik guruch kepagi ekstrakti, kremniy dioksidi</t>
+        </is>
+      </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>Взрослым — по 1 капсуле в день во время еды или запивая стаканом воды.</t>
+        </is>
+      </c>
+      <c r="S202" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 1 kapsula, ovqat vaqtida yoki bir stakan suv bilan.</t>
+        </is>
+      </c>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>Не использовать, если защитная плёнка повреждена или отсутствует. Хранить в недоступном для детей месте, в сухом и прохладном месте. Перед началом применения проконсультируйтесь с врачом.</t>
+        </is>
+      </c>
+      <c r="U202" t="inlineStr">
+        <is>
+          <t>Himoya pardasi shikastlangan yoki yoʻq boʻlsa, ishlatmang. Bolalar yeta olmaydigan, quruq va salqin joyda saqlang. Qoʻllashdan oldin shifokor bilan maslahatlashing.</t>
+        </is>
+      </c>
+      <c r="V202" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="W202" t="inlineStr">
+        <is>
+          <t>США</t>
+        </is>
+      </c>
+      <c r="X202" t="inlineStr">
+        <is>
+          <t>images/solaray-inositol-500.jpg</t>
+        </is>
+      </c>
+      <c r="Y202" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>solaray-tongkat-ali-400</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>solaray-tongkat-ali-400mg-60-vegcaps</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Solaray Tongkat Ali (Эврикома длиннолистная) 400 мг, 60 растительных капсул</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Solaray Tongkat Ali (Eurycoma longifolia) 400 mg, 60 oʻsimlik kapsulasi</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Травы и экстракты</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>Капсулы</t>
+        </is>
+      </c>
+      <c r="I203" t="n">
+        <v>400</v>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="K203" t="n">
+        <v>60</v>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>Корень эврикомы длиннолистной (тонгкат али) 400 мг — растительная поддержка.</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>Uzun bargli evrikoma ildizi (tongkat ali) 400 mg — oʻsimlik asosidagi yordam.</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>Solaray Tongkat Ali — корень эврикомы длиннолистной (Eurycoma longifolia), тропического растения из джунглей Индонезии, Малайзии и Вьетнама, который традиционно используется для растительной поддержки организма. Веганский продукт, сертификат Non-GMO Project Verified.</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>Solaray Tongkat Ali — Indoneziya, Malayziya va Vetnam oʻrmonlarida oʻsadigan tropik oʻsimlik — uzun bargli evrikoma (Eurycoma longifolia) ildizi; organizmni oʻsimlik asosida qoʻllab-quvvatlash uchun anʼanaviy ravishda ishlatiladi. Vegan mahsulot, Non-GMO Project Verified sertifikati.</t>
+        </is>
+      </c>
+      <c r="P203" t="inlineStr">
+        <is>
+          <t>1 капсула содержит: корень эврикомы длиннолистной (Eurycoma longifolia) — 400 мг; капсула из растительной целлюлозы, целлюлоза, стеарат магния, экстракт рисовых отрубей, диоксид кремния</t>
+        </is>
+      </c>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>1 kapsula tarkibida: uzun bargli evrikoma (Eurycoma longifolia) ildizi — 400 mg; oʻsimlik sellyulozasi kapsulasi, sellyuloza, magniy stearati, guruch kepagi ekstrakti, kremniy dioksidi</t>
+        </is>
+      </c>
+      <c r="R203" t="inlineStr">
+        <is>
+          <t>Взрослым — по 1 растительной капсуле 2 раза в день во время еды или запивая стаканом воды.</t>
+        </is>
+      </c>
+      <c r="S203" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 2 marta 1 tadan oʻsimlik kapsulasi, ovqat vaqtida yoki bir stakan suv bilan.</t>
+        </is>
+      </c>
+      <c r="T203" t="inlineStr">
+        <is>
+          <t>Не использовать, если защитная плёнка повреждена или отсутствует. Хранить в недоступном для детей месте, в сухом и прохладном месте. Перед началом применения проконсультируйтесь с врачом. Не принимать при беременности и кормлении грудью.</t>
+        </is>
+      </c>
+      <c r="U203" t="inlineStr">
+        <is>
+          <t>Himoya pardasi shikastlangan yoki yoʻq boʻlsa, ishlatmang. Bolalar yeta olmaydigan, quruq va salqin joyda saqlang. Qoʻllashdan oldin shifokor bilan maslahatlashing. Homiladorlik va emizish davrida qabul qilmang.</t>
+        </is>
+      </c>
+      <c r="V203" t="inlineStr">
+        <is>
+          <t>Solaray</t>
+        </is>
+      </c>
+      <c r="W203" t="inlineStr">
+        <is>
+          <t>США</t>
+        </is>
+      </c>
+      <c r="X203" t="inlineStr">
+        <is>
+          <t>images/solaray-tongkat-ali-400.jpg</t>
+        </is>
+      </c>
+      <c r="Y203" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>now-nac-600-selenium</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>now-nac-600mg-selenium-100-caps</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>NOW Foods NAC 600 мг с селеном, 100 капсул</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>NOW Foods NAC 600 mg selen bilan, 100 kapsula</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>NOW Foods</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Аминокислоты</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Антиоксиданты</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>Капсулы</t>
+        </is>
+      </c>
+      <c r="I204" t="n">
+        <v>600</v>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="K204" t="n">
+        <v>100</v>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>N-ацетилцистеин 600 мг с селеном — защита от свободных радикалов и здоровье клеток.</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>Selenli N-asetilsisteyin 600 mg — erkin radikallardan himoya va hujayra salomatligi.</t>
+        </is>
+      </c>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>NOW NAC — N-ацетилцистеин, стабильная форма заменимой аминокислоты цистеина, необходимой для образования глутатиона. В формулу добавлен селен — микроэлемент, участвующий в выработке важных ферментов. Защищает от свободных радикалов и поддерживает здоровье клеток. Без ГМО, кошерный и халяльный продукт.</t>
+        </is>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>NOW NAC — N-asetilsisteyin, glutation hosil boʻlishi uchun zarur boʻlgan almashinadigan aminokislota sisteinning barqaror shakli. Formulaga muhim fermentlar ishlab chiqarilishida ishtirok etuvchi mikroelement selen qoʻshilgan. Erkin radikallardan himoya qiladi va hujayra salomatligini qoʻllab-quvvatlaydi. GMOsiz, koshir va halol mahsulot.</t>
+        </is>
+      </c>
+      <c r="P204" t="inlineStr">
+        <is>
+          <t>1 капсула содержит: селен (элементарный, из L-селенометионина) — 25 мкг; N-ацетилцистеин (NAC) — 600 мг; гипромеллоза (целлюлозная капсула), стеариновая кислота (растительная), лимонная кислота, микрокристаллическая целлюлоза</t>
+        </is>
+      </c>
+      <c r="Q204" t="inlineStr">
+        <is>
+          <t>1 kapsula tarkibida: selen (elementar, L-selenometionindan) — 25 mkg; N-asetilsisteyin (NAC) — 600 mg; gipromelloza (sellyuloza kapsulasi), stearin kislotasi (oʻsimlik), limon kislotasi, mikrokristall sellyuloza</t>
+        </is>
+      </c>
+      <c r="R204" t="inlineStr">
+        <is>
+          <t>Взрослым — по 1 капсуле 2 раза в день.</t>
+        </is>
+      </c>
+      <c r="S204" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 2 marta 1 tadan kapsula.</t>
+        </is>
+      </c>
+      <c r="T204" t="inlineStr">
+        <is>
+          <t>Только для взрослых. Если вы беременны, кормите грудью, принимаете лекарства или у вас есть заболевания, проконсультируйтесь с врачом. Хранить в недоступном для детей месте. После вскрытия хранить в сухом и прохладном месте. Продукт может естественным образом менять цвет. На капсулах могут появиться крапинки — это не влияет на качество.</t>
+        </is>
+      </c>
+      <c r="U204" t="inlineStr">
+        <is>
+          <t>Faqat kattalar uchun. Homilador boʻlsangiz, emizayotgan boʻlsangiz, dori qabul qilsangiz yoki kasalligingiz boʻlsa, shifokor bilan maslahatlashing. Bolalar yeta olmaydigan joyda saqlang. Ochilgandan keyin quruq va salqin joyda saqlang. Mahsulot tabiiy ravishda rangini oʻzgartirishi mumkin. Kapsulalarda dogʻlar paydo boʻlishi mumkin — bu sifatga taʼsir qilmaydi.</t>
+        </is>
+      </c>
+      <c r="V204" t="inlineStr">
+        <is>
+          <t>NOW Foods</t>
+        </is>
+      </c>
+      <c r="W204" t="inlineStr">
+        <is>
+          <t>США</t>
+        </is>
+      </c>
+      <c r="X204" t="inlineStr">
+        <is>
+          <t>images/now-nac-600-selenium.jpg</t>
+        </is>
+      </c>
+      <c r="Y204" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>now-nac-1000</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>now-nac-1000mg-60-tabs</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>NOW Foods NAC 1000 мг, 60 таблеток</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>NOW Foods NAC 1000 mg, 60 tabletka</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>NOW Foods</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Аминокислоты</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Пищеварение и печень</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Таблетки</t>
+        </is>
+      </c>
+      <c r="I205" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="K205" t="n">
+        <v>60</v>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>N-ацетилцистеин 1000 мг — защита от свободных радикалов, иммунитет и здоровье печени.</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>N-asetilsisteyin 1000 mg — erkin radikallardan himoya, immunitet va jigar salomatligi.</t>
+        </is>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>NOW NAC 1000 — N-ацетилцистеин, стабильная форма аминокислоты цистеина, поддерживающая образование глутатиона — мощного соединения, нейтрализующего свободные радикалы. Поддерживает иммунную систему и здоровье печени. Подходит для вегетарианцев и веганов, без ГМО.</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>NOW NAC 1000 — sisteyin aminokislotasining barqaror shakli boʻlgan N-asetilsisteyin; erkin radikallarni zararsizlantiruvchi kuchli birikma — glutation hosil boʻlishini qoʻllab-quvvatlaydi. Immun tizimi va jigar salomatligini qoʻllab-quvvatlaydi. Vegetarianlar va veganlar uchun mos, GMOsiz.</t>
+        </is>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>1 таблетка содержит: N-ацетилцистеин (NAC) — 1000 мг; микрокристаллическая целлюлоза, гидроксипропилцеллюлоза, стеариновая кислота (растительная), кроскармеллоза натрия, оболочка (гипромеллоза, лецитин подсолнечника, триэтилцитрат), диоксид кремния</t>
+        </is>
+      </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>1 tabletka tarkibida: N-asetilsisteyin (NAC) — 1000 mg; mikrokristall sellyuloza, gidroksipropilsellyuloza, stearin kislotasi (oʻsimlik), natriy kroskarmelloza, qobiq (gipromelloza, kungaboqar lesitini, trietilsitrat), kremniy dioksidi</t>
+        </is>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>Взрослым — по 1 таблетке 1–3 раза в день.</t>
+        </is>
+      </c>
+      <c r="S205" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 1–3 marta 1 tadan tabletka.</t>
+        </is>
+      </c>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>Только для взрослых. Перед применением при беременности, кормлении грудью, приёме лекарств (особенно нитроглицерина) или наличии заболеваний проконсультируйтесь с врачом. Хранить в недоступном для детей месте. После вскрытия хранить в сухом и прохладном месте. Продукт может естественным образом менять цвет.</t>
+        </is>
+      </c>
+      <c r="U205" t="inlineStr">
+        <is>
+          <t>Faqat kattalar uchun. Homiladorlik, emizish davrida, dori (ayniqsa nitrogliserin) qabul qilganda yoki kasallik mavjud boʻlganda qoʻllashdan oldin shifokor bilan maslahatlashing. Bolalar yeta olmaydigan joyda saqlang. Ochilgandan keyin quruq va salqin joyda saqlang. Mahsulot tabiiy ravishda rangini oʻzgartirishi mumkin.</t>
+        </is>
+      </c>
+      <c r="V205" t="inlineStr">
+        <is>
+          <t>NOW Foods</t>
+        </is>
+      </c>
+      <c r="W205" t="inlineStr">
+        <is>
+          <t>США</t>
+        </is>
+      </c>
+      <c r="X205" t="inlineStr">
+        <is>
+          <t>images/now-nac-1000.jpg</t>
+        </is>
+      </c>
+      <c r="Y205" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>now-coq10-100-hawthorn</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>now-coq10-100mg-hawthorn-30-vcaps</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>NOW Foods CoQ10 100 мг с боярышником, 30 растительных капсул</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>NOW Foods CoQ10 100 mg andoʻz bilan, 30 oʻsimlik kapsulasi</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>NOW Foods</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Антиоксиданты</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Капсулы</t>
+        </is>
+      </c>
+      <c r="I206" t="n">
+        <v>100</v>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="K206" t="n">
+        <v>30</v>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>Коэнзим Q10 100 мг с ягодами боярышника для сердца и выработки клеточной энергии.</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>Yurak va hujayra energiyasi ishlab chiqarilishi uchun andoʻz mevali koenzim Q10 100 mg.</t>
+        </is>
+      </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>NOW CoQ10 — коэнзим Q10, витаминоподобное соединение, играющее ключевую роль в выработке клеточной энергии. Больше всего его в сердце, печени и почках, а с возрастом собственная выработка снижается. В формулу добавлены ягоды боярышника. Поддерживает здоровье сердечно-сосудистой системы. Для вегетарианцев и веганов, сертификат Non-GMO Project Verified.</t>
+        </is>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>NOW CoQ10 — hujayra energiyasi ishlab chiqarilishida muhim rol oʻynaydigan vitaminga oʻxshash birikma — koenzim Q10. Eng koʻp yurak, jigar va buyraklarda boʻladi, yosh oʻtgan sari oʻz ishlab chiqarilishi kamayadi. Formulaga andoʻz mevalari qoʻshilgan. Yurak-qon tomir tizimi salomatligini qoʻllab-quvvatlaydi. Vegetarianlar va veganlar uchun, Non-GMO Project Verified sertifikati.</t>
+        </is>
+      </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>1 капсула содержит: коэнзим Q10 (CoQ10) — 100 мг; ягоды боярышника (Crataegus laevigata и/или monogyna) — 400 мг; гипромеллоза (целлюлозная капсула)</t>
+        </is>
+      </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>1 kapsula tarkibida: koenzim Q10 (CoQ10) — 100 mg; andoʻz mevalari (Crataegus laevigata va/yoki monogyna) — 400 mg; gipromelloza (sellyuloza kapsulasi)</t>
+        </is>
+      </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>Взрослым — по 1 капсуле в день во время приёма жиросодержащей пищи.</t>
+        </is>
+      </c>
+      <c r="S206" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 1 kapsula, yogʻli ovqat bilan birga.</t>
+        </is>
+      </c>
+      <c r="T206" t="inlineStr">
+        <is>
+          <t>Только для взрослых. Если вы беременны, кормите грудью, принимаете лекарства или у вас есть заболевания, проконсультируйтесь с врачом. Хранить в недоступном для детей месте. После вскрытия хранить в сухом и прохладном месте. Продукт может естественным образом менять цвет.</t>
+        </is>
+      </c>
+      <c r="U206" t="inlineStr">
+        <is>
+          <t>Faqat kattalar uchun. Homilador boʻlsangiz, emizayotgan boʻlsangiz, dori qabul qilsangiz yoki kasalligingiz boʻlsa, shifokor bilan maslahatlashing. Bolalar yeta olmaydigan joyda saqlang. Ochilgandan keyin quruq va salqin joyda saqlang. Mahsulot tabiiy ravishda rangini oʻzgartirishi mumkin.</t>
+        </is>
+      </c>
+      <c r="V206" t="inlineStr">
+        <is>
+          <t>NOW Foods</t>
+        </is>
+      </c>
+      <c r="W206" t="inlineStr">
+        <is>
+          <t>США</t>
+        </is>
+      </c>
+      <c r="X206" t="inlineStr">
+        <is>
+          <t>images/now-coq10-100-hawthorn.jpg</t>
+        </is>
+      </c>
+      <c r="Y206" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>ecovita-magnesium-glycinate-360</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>ecovita-magnesium-glycinate-360mg-120</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>ECOVITA Magnesium Glycinate 360 мг, 120 капсул</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>ECOVITA Magnesium Glycinate 360 mg, 120 kapsula</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>ECOVITA</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Минералы</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Нервная система и сон</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Капсулы</t>
+        </is>
+      </c>
+      <c r="I207" t="n">
+        <v>360</v>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="K207" t="n">
+        <v>120</v>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>Магний в форме бисглицината — снижает мышечное напряжение, поддерживает нервную систему и отдых.</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>Bisglitsinat shaklidagi magniy — mushaklar zoʻriqishini kamaytiradi, asab tizimi va dam olishni qoʻllab-quvvatlaydi.</t>
+        </is>
+      </c>
+      <c r="N207" t="inlineStr">
+        <is>
+          <t>ECOVITA Magnesium Glycinate (магний хелат усиленный) — магний в виде бисглицината, хорошо усваиваемой хелатной формы. Помогает снижать мышечное напряжение, поддерживает здоровье нервной системы и способствует полноценному отдыху. Дополнительный источник магния. Халяль.</t>
+        </is>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>ECOVITA Magnesium Glycinate (kuchaytirilgan magniy xelat) — yaxshi oʻzlashadigan xelat shakli boʻlgan bisglitsinat koʻrinishidagi magniy. Mushaklar zoʻriqishini kamaytirishga, asab tizimi salomatligini qoʻllab-quvvatlashga va toʻliq dam olishga yordam beradi. Magniyning qoʻshimcha manbai. Halol.</t>
+        </is>
+      </c>
+      <c r="P207" t="inlineStr">
+        <is>
+          <t>3 капсулы содержат: магния бисглицинат — 1800 мг; элементарный магний — 360 мг; микрокристаллическая целлюлоза (носитель), диоксид кремния (антислеживатель), капсула (желатин или гидроксипропилметилцеллюлоза)</t>
+        </is>
+      </c>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>3 kapsula tarkibida: magniy bisglitsinat — 1800 mg; elementar magniy — 360 mg; mikrokristall sellyuloza (tashuvchi), kremniy dioksidi (qotib qolishga qarshi), kapsula (jelatin yoki gidroksipropilmetilsellyuloza)</t>
+        </is>
+      </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>Взрослым — по 3–4 капсулы в день во время приёма пищи. Продолжительность приёма — 1 месяц, при необходимости курс можно повторить.</t>
+        </is>
+      </c>
+      <c r="S207" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 3–4 kapsula, ovqat vaqtida. Qabul muddati — 1 oy, zarur boʻlsa kursni takrorlash mumkin.</t>
+        </is>
+      </c>
+      <c r="T207" t="inlineStr">
+        <is>
+          <t>Индивидуальная непереносимость компонентов, беременность, период лактации, возраст до 18 лет. Перед применением проконсультируйтесь с врачом. Хранить в сухом, прохладном, защищённом от прямых солнечных лучей и недоступном для детей месте при температуре не выше 25°C и относительной влажности не более 75%, в закрытой неповреждённой упаковке. Срок годности — 2 года.</t>
+        </is>
+      </c>
+      <c r="U207" t="inlineStr">
+        <is>
+          <t>Tarkibiy qismlarga individual toʻqnashmovchilik, homiladorlik, laktatsiya davri, 18 yoshgacha. Qoʻllashdan oldin shifokor bilan maslahatlashing. Quruq, salqin, toʻgʻridan-toʻgʻri quyosh nuridan himoyalangan, bolalar yeta olmaydigan joyda, 25°C dan yuqori boʻlmagan haroratda va nisbiy namlik 75% dan oshmagan sharoitda, yopiq butun qadoqda saqlang. Yaroqlilik muddati — 2 yil.</t>
+        </is>
+      </c>
+      <c r="V207" t="inlineStr">
+        <is>
+          <t>ECOVITA</t>
+        </is>
+      </c>
+      <c r="W207" t="inlineStr">
+        <is>
+          <t>Россия</t>
+        </is>
+      </c>
+      <c r="X207" t="inlineStr">
+        <is>
+          <t>images/ecovita-magnesium-glycinate-360.jpg</t>
+        </is>
+      </c>
+      <c r="Y207" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>ecovita-magnesium-malate-200</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>ecovita-magnesium-malate-200mg-60</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>ECOVITA Magnesium Malate 200 мг, 60 капсул</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>ECOVITA Magnesium Malate 200 mg, 60 kapsula</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>ECOVITA</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Минералы</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Капсулы</t>
+        </is>
+      </c>
+      <c r="I208" t="n">
+        <v>200</v>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="K208" t="n">
+        <v>60</v>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>Малат магния — клеточная энергия, снижение усталости и поддержка мышц.</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>Magniy malat — hujayra energiyasi, charchoqni kamaytirish va mushaklarni qoʻllab-quvvatlash.</t>
+        </is>
+      </c>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>ECOVITA Magnesium Malate — магний в форме малата (соли яблочной кислоты). Поддерживает выработку клеточной энергии, помогает снижать усталость и утомляемость, поддерживает мышечную функцию. Дополнительный источник магния. Халяль.</t>
+        </is>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>ECOVITA Magnesium Malate — malat (olma kislotasi tuzi) shaklidagi magniy. Hujayra energiyasi ishlab chiqarilishini qoʻllab-quvvatlaydi, charchoq va holsizlikni kamaytirishga yordam beradi, mushak funksiyasini qoʻllab-quvvatlaydi. Magniyning qoʻshimcha manbai. Halol.</t>
+        </is>
+      </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t>2 капсулы содержат: магния малат — 1250 мг; элементарный магний — 200 мг; микрокристаллическая целлюлоза (носитель), желатиновая капсула</t>
+        </is>
+      </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>2 kapsula tarkibida: magniy malat — 1250 mg; elementar magniy — 200 mg; mikrokristall sellyuloza (tashuvchi), jelatin kapsulasi</t>
+        </is>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>Взрослым — по 2 капсулы в день во время приёма пищи. Продолжительность приёма — 1 месяц, при необходимости курс можно повторить.</t>
+        </is>
+      </c>
+      <c r="S208" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 2 kapsula, ovqat vaqtida. Qabul muddati — 1 oy, zarur boʻlsa kursni takrorlash mumkin.</t>
+        </is>
+      </c>
+      <c r="T208" t="inlineStr">
+        <is>
+          <t>Индивидуальная непереносимость компонентов, беременность, период лактации, возраст до 18 лет. Перед применением проконсультируйтесь с врачом. Хранить в сухом, прохладном, защищённом от прямых солнечных лучей и недоступном для детей месте при температуре не выше 25°C и относительной влажности не более 75%, в закрытой неповреждённой упаковке. Срок годности — 2 года.</t>
+        </is>
+      </c>
+      <c r="U208" t="inlineStr">
+        <is>
+          <t>Tarkibiy qismlarga individual toʻqnashmovchilik, homiladorlik, laktatsiya davri, 18 yoshgacha. Qoʻllashdan oldin shifokor bilan maslahatlashing. Quruq, salqin, toʻgʻridan-toʻgʻri quyosh nuridan himoyalangan, bolalar yeta olmaydigan joyda, 25°C dan yuqori boʻlmagan haroratda va nisbiy namlik 75% dan oshmagan sharoitda, yopiq butun qadoqda saqlang. Yaroqlilik muddati — 2 yil.</t>
+        </is>
+      </c>
+      <c r="V208" t="inlineStr">
+        <is>
+          <t>ECOVITA</t>
+        </is>
+      </c>
+      <c r="W208" t="inlineStr">
+        <is>
+          <t>Россия</t>
+        </is>
+      </c>
+      <c r="X208" t="inlineStr">
+        <is>
+          <t>images/ecovita-magnesium-malate-200.jpg</t>
+        </is>
+      </c>
+      <c r="Y208" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>ecovita-alpha-lipoic-acid</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>ecovita-alpha-lipoic-acid-100mg-60</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>ECOVITA Alpha Lipoic Acid 100 мг, 60 капсул</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>ECOVITA Alpha Lipoic Acid 100 mg, 60 kapsula</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>ECOVITA</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Антиоксиданты</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Пищеварение и печень</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Капсулы</t>
+        </is>
+      </c>
+      <c r="I209" t="n">
+        <v>100</v>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="K209" t="n">
+        <v>60</v>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>Альфа-липоевая кислота 100 мг — антиоксидантная защита, детокс и здоровье печени.</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>Alfa-lipoy kislotasi 100 mg — antioksidant himoya, detoks va jigar salomatligi.</t>
+        </is>
+      </c>
+      <c r="N209" t="inlineStr">
+        <is>
+          <t>ECOVITA Alpha Lipoic Acid — дополнительный источник альфа-липоевой кислоты, мощного антиоксиданта. Поддерживает детоксикацию и здоровье печени, обеспечивает антиоксидантную защиту и поддерживает здоровый метаболизм при снижении веса. Халяль.</t>
+        </is>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>ECOVITA Alpha Lipoic Acid — kuchli antioksidant boʻlgan alfa-lipoy kislotasining qoʻshimcha manbai. Detoksikatsiya va jigar salomatligini qoʻllab-quvvatlaydi, antioksidant himoyani taʼminlaydi va ozish paytida sogʻlom metabolizmni qoʻllab-quvvatlaydi. Halol.</t>
+        </is>
+      </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t>1 капсула содержит: альфа-липоевая кислота — 100 мг; микрокристаллическая целлюлоза (носитель), желатиновая капсула</t>
+        </is>
+      </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>1 kapsula tarkibida: alfa-lipoy kislotasi — 100 mg; mikrokristall sellyuloza (tashuvchi), jelatin kapsulasi</t>
+        </is>
+      </c>
+      <c r="R209" t="inlineStr">
+        <is>
+          <t>Взрослым — по 1 капсуле в день во время еды или по рекомендации врача. Продолжительность приёма — 1 месяц, при необходимости курс можно повторить.</t>
+        </is>
+      </c>
+      <c r="S209" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 1 kapsula, ovqat vaqtida yoki shifokor tavsiyasiga koʻra. Qabul muddati — 1 oy, zarur boʻlsa kursni takrorlash mumkin.</t>
+        </is>
+      </c>
+      <c r="T209" t="inlineStr">
+        <is>
+          <t>Индивидуальная непереносимость компонентов, беременность, период лактации, возраст до 18 лет. Перед применением проконсультируйтесь с врачом. Хранить в сухом, прохладном, защищённом от прямых солнечных лучей и недоступном для детей месте при температуре не выше 25°C и относительной влажности не более 75%, в закрытой неповреждённой упаковке. Срок годности — 2 года.</t>
+        </is>
+      </c>
+      <c r="U209" t="inlineStr">
+        <is>
+          <t>Tarkibiy qismlarga individual toʻqnashmovchilik, homiladorlik, laktatsiya davri, 18 yoshgacha. Qoʻllashdan oldin shifokor bilan maslahatlashing. Quruq, salqin, toʻgʻridan-toʻgʻri quyosh nuridan himoyalangan, bolalar yeta olmaydigan joyda, 25°C dan yuqori boʻlmagan haroratda va nisbiy namlik 75% dan oshmagan sharoitda, yopiq butun qadoqda saqlang. Yaroqlilik muddati — 2 yil.</t>
+        </is>
+      </c>
+      <c r="V209" t="inlineStr">
+        <is>
+          <t>ECOVITA</t>
+        </is>
+      </c>
+      <c r="W209" t="inlineStr">
+        <is>
+          <t>Россия</t>
+        </is>
+      </c>
+      <c r="X209" t="inlineStr">
+        <is>
+          <t>images/ecovita-alpha-lipoic-acid.jpg</t>
+        </is>
+      </c>
+      <c r="Y209" t="inlineStr">
+        <is>
+          <t>опубликован</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>ecovita-5-htp-b6</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>ecovita-5-htp-vitamin-b6-200mg-60</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>ECOVITA 5-HTP + Vitamin B6 200 мг + 2 мг, 60 капсул</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>ECOVITA 5-HTP + Vitamin B6 200 mg + 2 mg, 60 kapsula</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>ECOVITA</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Нервная система и сон</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Аминокислоты</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Капсулы</t>
+        </is>
+      </c>
+      <c r="I210" t="n">
+        <v>200</v>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>мг</t>
+        </is>
+      </c>
+      <c r="K210" t="n">
+        <v>60</v>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>5-гидрокситриптофан с витамином B6 — спокойствие, качество сна и выработка серотонина.</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>B6 vitaminli 5-gidroksitriptofan — xotirjamlik, uyqu sifati va serotonin ishlab chiqarilishi.</t>
+        </is>
+      </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>ECOVITA 5-HTP + Vitamin B6 — комплекс 5-гидрокситриптофана и витамина B6. Способствует спокойствию и эмоциональному комфорту, улучшению качества сна и поддерживает естественную выработку серотонина. Дополнительный источник витамина B6. Халяль.</t>
+        </is>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>ECOVITA 5-HTP + Vitamin B6 — 5-gidroksitriptofan va B6 vitamini kompleksi. Xotirjamlik va hissiy qulaylikka, uyqu sifatini yaxshilashga yordam beradi hamda serotoninning tabiiy ishlab chiqarilishini qoʻllab-quvvatlaydi. B6 vitaminining qoʻshimcha manbai. Halol.</t>
+        </is>
+      </c>
+      <c r="P210" t="inlineStr">
+        <is>
+          <t>2 капсулы содержат: 5-гидрокситриптофан (5-HTP) — 200 мг; витамин B6 (пиридоксина гидрохлорид) — 2 мг; микрокристаллическая целлюлоза (носитель), мальтодекстрин (носитель), диоксид кремния (антислеживатель), желатиновая капсула</t>
+        </is>
+      </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>2 kapsula tarkibida: 5-gidroksitriptofan (5-HTP) — 200 mg; vitamin B6 (piridoksin gidroxlorid) — 2 mg; mikrokristall sellyuloza (tashuvchi), maltodekstrin (tashuvchi), kremniy dioksidi (qotib qolishga qarshi), jelatin kapsulasi</t>
+        </is>
+      </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>Взрослым — по 1 капсуле 2 раза в день. Продолжительность приёма — 1 месяц, при необходимости курс можно повторить.</t>
+        </is>
+      </c>
+      <c r="S210" t="inlineStr">
+        <is>
+          <t>Kattalar uchun — kuniga 2 marta 1 tadan kapsula. Qabul muddati — 1 oy, zarur boʻlsa kursni takrorlash mumkin.</t>
+        </is>
+      </c>
+      <c r="T210" t="inlineStr">
+        <is>
+          <t>Индивидуальная непереносимость компонентов, беременность, период лактации. Перед применением проконсультируйтесь с врачом. Хранить в сухом, прохладном, защищённом от прямых солнечных лучей и недоступном для детей месте при температуре не выше 25°C и относительной влажности не более 75%, в закрытой неповреждённой упаковке. Срок годности — 2 года.</t>
+        </is>
+      </c>
+      <c r="U210" t="inlineStr">
+        <is>
+          <t>Tarkibiy qismlarga individual toʻqnashmovchilik, homiladorlik, laktatsiya davri. Qoʻllashdan oldin shifokor bilan maslahatlashing. Quruq, salqin, toʻgʻridan-toʻgʻri quyosh nuridan himoyalangan, bolalar yeta olmaydigan joyda, 25°C dan yuqori boʻlmagan haroratda va nisbiy namlik 75% dan oshmagan sharoitda, yopiq butun qadoqda saqlang. Yaroqlilik muddati — 2 yil.</t>
+        </is>
+      </c>
+      <c r="V210" t="inlineStr">
+        <is>
+          <t>ECOVITA</t>
+        </is>
+      </c>
+      <c r="W210" t="inlineStr">
+        <is>
+          <t>Россия</t>
+        </is>
+      </c>
+      <c r="X210" t="inlineStr">
+        <is>
+          <t>images/ecovita-5-htp-b6.jpg</t>
+        </is>
+      </c>
+      <c r="Y210" t="inlineStr">
         <is>
           <t>опубликован</t>
         </is>
@@ -25285,7 +26987,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3">
@@ -25295,7 +26997,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -25315,7 +27017,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -25335,7 +27037,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">

</xml_diff>